<commit_message>
Universal calibration ledger: replace ad-hoc LEDGER with security-agnostic schema (instrument + asset_class, anchor/horizon/cycle/reanchor, P5-P95, relative touch bands, full grade-time columns + touch-hit flags); log PHDC + TMGH anchors with grades pending; update ledger.html + app.js consumers; add matching Calibration Ledger tab to PHDC & TMGH study Excel models (0 formula errors). Canonical default for all future studies, any exchange/asset class.
</commit_message>
<xml_diff>
--- a/files/PHDC_Valuation_Study_11-06-2026_public.xlsx
+++ b/files/PHDC_Valuation_Study_11-06-2026_public.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Valuation" sheetId="10" state="visible" r:id="rId12"/>
     <sheet name="Monte Carlo" sheetId="11" state="visible" r:id="rId13"/>
     <sheet name="Sensitivity" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Calibration Ledger" sheetId="13" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="408">
   <si>
     <t xml:space="preserve">READ FIRST — DISCLOSURE &amp; DISCLAIMER · PHDC VALUATION MODEL (EDUCATIONAL)</t>
   </si>
@@ -1111,6 +1112,150 @@
   </si>
   <si>
     <t xml:space="preserve">Price level →</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CALIBRATION LEDGER — universal, security-agnostic forecast record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every published forecast is logged here at its anchor and graded when the horizon matures. Schema is asset-class-agnostic (equity / metal / other) and identical across all studies. Grade-time columns stay blank until grade_date, then carry the realized outcome.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANCHOR (logged at publication)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREDICTED PERCENTILES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOUCH BANDS — P(touch ±x% from anchor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRADE-TIME (blank until grade_date)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instrument</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anchor price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ccy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grade date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cycle #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-anchor from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P50 (median)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch +5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch +10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch +15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch +20%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch −5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touch −10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realized close</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realized high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realized low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In 90%?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In 50%?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realized quantile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median err</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit +5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit +10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit +15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit +20%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit −5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hit −10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PHDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T+20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-06-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T+60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status is derived: a row is OPEN until realized_close is entered, then GRADED. in_90 / in_50 = realized_close within the P5–P95 / P25–P75 band. realized_quantile = empirical position of the realized close in the predicted distribution (0–1). median_err = realized_close − P50. Touch-hit flags record whether each ±x% level was reached within the horizon window.</t>
   </si>
 </sst>
 </file>
@@ -1131,7 +1276,7 @@
     <numFmt numFmtId="174" formatCode="0.00;[RED]\-0.00"/>
     <numFmt numFmtId="175" formatCode="0.00\x"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1304,8 +1449,32 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF1B5E5E"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF6B6B6B"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FF6B6B6B"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1336,8 +1505,14 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC98A2D"/>
+        <bgColor rgb="FFFF8080"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1357,6 +1532,15 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1386,7 +1570,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="95">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1731,6 +1915,42 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1756,7 +1976,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF1B5E5E"/>
-      <rgbColor rgb="FFB0B0B0"/>
+      <rgbColor rgb="FFBFBFBF"/>
       <rgbColor rgb="FF6B7676"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -1786,10 +2006,10 @@
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFC98A2D"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF6B6B6B"/>
+      <rgbColor rgb="FFB0B0B0"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF2A8F8F"/>
       <rgbColor rgb="FF003300"/>
@@ -3995,6 +4215,351 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:AG9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="10" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="22" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="24" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="28" style="0" width="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="86" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="87" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="88" t="s">
+        <v>362</v>
+      </c>
+      <c r="B4" s="88"/>
+      <c r="C4" s="88"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="89" t="s">
+        <v>363</v>
+      </c>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="89"/>
+      <c r="N4" s="89"/>
+      <c r="O4" s="89" t="s">
+        <v>364</v>
+      </c>
+      <c r="P4" s="89"/>
+      <c r="Q4" s="89"/>
+      <c r="R4" s="89"/>
+      <c r="S4" s="89"/>
+      <c r="T4" s="89"/>
+      <c r="U4" s="90" t="s">
+        <v>365</v>
+      </c>
+      <c r="V4" s="90"/>
+      <c r="W4" s="90"/>
+      <c r="X4" s="90"/>
+      <c r="Y4" s="90"/>
+      <c r="Z4" s="90"/>
+      <c r="AA4" s="90"/>
+      <c r="AB4" s="90"/>
+      <c r="AC4" s="90"/>
+      <c r="AD4" s="90"/>
+      <c r="AE4" s="90"/>
+      <c r="AF4" s="90"/>
+      <c r="AG4" s="90"/>
+    </row>
+    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="s">
+        <v>366</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>367</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>368</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>369</v>
+      </c>
+      <c r="E5" s="26" t="s">
+        <v>370</v>
+      </c>
+      <c r="F5" s="26" t="s">
+        <v>326</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>371</v>
+      </c>
+      <c r="H5" s="26" t="s">
+        <v>372</v>
+      </c>
+      <c r="I5" s="26" t="s">
+        <v>373</v>
+      </c>
+      <c r="J5" s="26" t="s">
+        <v>374</v>
+      </c>
+      <c r="K5" s="26" t="s">
+        <v>375</v>
+      </c>
+      <c r="L5" s="26" t="s">
+        <v>376</v>
+      </c>
+      <c r="M5" s="26" t="s">
+        <v>377</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>378</v>
+      </c>
+      <c r="O5" s="26" t="s">
+        <v>379</v>
+      </c>
+      <c r="P5" s="26" t="s">
+        <v>380</v>
+      </c>
+      <c r="Q5" s="26" t="s">
+        <v>381</v>
+      </c>
+      <c r="R5" s="26" t="s">
+        <v>382</v>
+      </c>
+      <c r="S5" s="26" t="s">
+        <v>383</v>
+      </c>
+      <c r="T5" s="26" t="s">
+        <v>384</v>
+      </c>
+      <c r="U5" s="26" t="s">
+        <v>385</v>
+      </c>
+      <c r="V5" s="26" t="s">
+        <v>386</v>
+      </c>
+      <c r="W5" s="26" t="s">
+        <v>387</v>
+      </c>
+      <c r="X5" s="26" t="s">
+        <v>388</v>
+      </c>
+      <c r="Y5" s="26" t="s">
+        <v>389</v>
+      </c>
+      <c r="Z5" s="26" t="s">
+        <v>390</v>
+      </c>
+      <c r="AA5" s="26" t="s">
+        <v>391</v>
+      </c>
+      <c r="AB5" s="26" t="s">
+        <v>392</v>
+      </c>
+      <c r="AC5" s="26" t="s">
+        <v>393</v>
+      </c>
+      <c r="AD5" s="26" t="s">
+        <v>394</v>
+      </c>
+      <c r="AE5" s="26" t="s">
+        <v>395</v>
+      </c>
+      <c r="AF5" s="26" t="s">
+        <v>396</v>
+      </c>
+      <c r="AG5" s="26" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="91" t="s">
+        <v>398</v>
+      </c>
+      <c r="B6" s="91" t="s">
+        <v>399</v>
+      </c>
+      <c r="C6" s="91" t="s">
+        <v>400</v>
+      </c>
+      <c r="D6" s="92" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E6" s="91" t="s">
+        <v>401</v>
+      </c>
+      <c r="F6" s="91" t="s">
+        <v>402</v>
+      </c>
+      <c r="G6" s="91" t="s">
+        <v>403</v>
+      </c>
+      <c r="H6" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="91" t="s">
+        <v>404</v>
+      </c>
+      <c r="J6" s="92" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="K6" s="92" t="n">
+        <v>13.42</v>
+      </c>
+      <c r="L6" s="92" t="n">
+        <v>14.92</v>
+      </c>
+      <c r="M6" s="92" t="n">
+        <v>16.56</v>
+      </c>
+      <c r="N6" s="92" t="n">
+        <v>19.32</v>
+      </c>
+      <c r="O6" s="93" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="P6" s="93" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="Q6" s="93" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="R6" s="93" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="S6" s="93" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="T6" s="93" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="U6" s="91"/>
+      <c r="V6" s="91"/>
+      <c r="W6" s="91"/>
+      <c r="X6" s="91"/>
+      <c r="Y6" s="91"/>
+      <c r="Z6" s="91"/>
+      <c r="AA6" s="91"/>
+      <c r="AB6" s="91"/>
+      <c r="AC6" s="91"/>
+      <c r="AD6" s="91"/>
+      <c r="AE6" s="91"/>
+      <c r="AF6" s="91"/>
+      <c r="AG6" s="91"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="91" t="s">
+        <v>398</v>
+      </c>
+      <c r="B7" s="91" t="s">
+        <v>399</v>
+      </c>
+      <c r="C7" s="91" t="s">
+        <v>400</v>
+      </c>
+      <c r="D7" s="92" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="E7" s="91" t="s">
+        <v>401</v>
+      </c>
+      <c r="F7" s="91" t="s">
+        <v>405</v>
+      </c>
+      <c r="G7" s="91" t="s">
+        <v>406</v>
+      </c>
+      <c r="H7" s="91" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="91" t="s">
+        <v>404</v>
+      </c>
+      <c r="J7" s="92" t="n">
+        <v>10.18</v>
+      </c>
+      <c r="K7" s="92" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="L7" s="92" t="n">
+        <v>15.83</v>
+      </c>
+      <c r="M7" s="92" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N7" s="92" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="O7" s="93" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P7" s="93" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="Q7" s="93" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="R7" s="93" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="S7" s="93" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="T7" s="93" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="U7" s="91"/>
+      <c r="V7" s="91"/>
+      <c r="W7" s="91"/>
+      <c r="X7" s="91"/>
+      <c r="Y7" s="91"/>
+      <c r="Z7" s="91"/>
+      <c r="AA7" s="91"/>
+      <c r="AB7" s="91"/>
+      <c r="AC7" s="91"/>
+      <c r="AD7" s="91"/>
+      <c r="AE7" s="91"/>
+      <c r="AF7" s="91"/>
+      <c r="AG7" s="91"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="94" t="s">
+        <v>407</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>